<commit_message>
add 1 case for NEO3-17020
add 1 case for NEO3-17020
</commit_message>
<xml_diff>
--- a/Custom_Quick Chip Mode_TW/0_Tool+doc/QuickChip test list.xlsx
+++ b/Custom_Quick Chip Mode_TW/0_Tool+doc/QuickChip test list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26529"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\test_tree\Custom_Quick Chip Mode_TW\0_Tool+doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC44167-C260-4F3A-B082-8401EC71F77A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF91D2C-16E6-4370-B4FF-D826F7F536FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="960" yWindow="2340" windowWidth="15900" windowHeight="12495" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="255" yWindow="780" windowWidth="16785" windowHeight="13845" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="163">
   <si>
     <t>Item</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -3845,6 +3845,14 @@
     <t>Tag DFEC4F: bootup notification</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>QCM014-1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fallback to MSR: enable/ disable</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -3853,7 +3861,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="m&quot;月&quot;d&quot;日&quot;"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="15">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -4484,8 +4492,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E51"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:E52"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="16" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="51.625" style="19" bestFit="1" customWidth="1"/>
@@ -4495,7 +4503,7 @@
     <col min="6" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5">
       <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
@@ -4509,7 +4517,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="63" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="63">
       <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
@@ -4523,7 +4531,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="127.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="127.5">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
@@ -4537,7 +4545,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5">
       <c r="A4" s="8" t="s">
         <v>30</v>
       </c>
@@ -4551,7 +4559,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="63.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="63.75">
       <c r="A5" s="6" t="s">
         <v>32</v>
       </c>
@@ -4565,7 +4573,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="111.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="111.75">
       <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
@@ -4582,7 +4590,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="33">
       <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
@@ -4596,7 +4604,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="16.5">
       <c r="A8" s="6" t="s">
         <v>5</v>
       </c>
@@ -4610,7 +4618,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="78.75">
       <c r="A9" s="26" t="s">
         <v>100</v>
       </c>
@@ -4624,7 +4632,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="63" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="63">
       <c r="A10" s="6" t="s">
         <v>5</v>
       </c>
@@ -4638,7 +4646,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5">
       <c r="A11" s="6" t="s">
         <v>5</v>
       </c>
@@ -4652,545 +4660,559 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>29</v>
+    <row r="12" spans="1:5">
+      <c r="A12" s="6" t="s">
+        <v>5</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>47</v>
+        <v>162</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>62</v>
+        <v>161</v>
       </c>
       <c r="D12" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="B13" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="C13" s="25" t="s">
-        <v>63</v>
+    <row r="13" spans="1:5" ht="31.5">
+      <c r="A13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>62</v>
       </c>
       <c r="D13" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="36" t="s">
+    <row r="14" spans="1:5" ht="31.5">
+      <c r="A14" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="31.5">
+      <c r="A15" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="32" t="s">
+      <c r="B15" s="32" t="s">
         <v>134</v>
       </c>
-      <c r="C14" s="35" t="s">
+      <c r="C15" s="35" t="s">
         <v>106</v>
-      </c>
-      <c r="D14" s="34" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="37"/>
-      <c r="B15" s="32" t="s">
-        <v>135</v>
-      </c>
-      <c r="C15" s="35" t="s">
-        <v>107</v>
       </c>
       <c r="D15" s="34" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="38"/>
+    <row r="16" spans="1:5" ht="31.5">
+      <c r="A16" s="37"/>
       <c r="B16" s="32" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="C16" s="35" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D16" s="34" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="36" t="s">
-        <v>5</v>
-      </c>
+    <row r="17" spans="1:4" ht="31.5">
+      <c r="A17" s="38"/>
       <c r="B17" s="32" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C17" s="35" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D17" s="34" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="37"/>
+    <row r="18" spans="1:4" ht="31.5">
+      <c r="A18" s="36" t="s">
+        <v>5</v>
+      </c>
       <c r="B18" s="32" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C18" s="35" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D18" s="34" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="38"/>
+    <row r="19" spans="1:4" ht="31.5">
+      <c r="A19" s="37"/>
       <c r="B19" s="32" t="s">
+        <v>130</v>
+      </c>
+      <c r="C19" s="35" t="s">
+        <v>110</v>
+      </c>
+      <c r="D19" s="34" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="31.5">
+      <c r="A20" s="38"/>
+      <c r="B20" s="32" t="s">
         <v>131</v>
       </c>
-      <c r="C19" s="35" t="s">
+      <c r="C20" s="35" t="s">
         <v>125</v>
       </c>
-      <c r="D19" s="34"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="36" t="s">
+      <c r="D20" s="34"/>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="B20" s="32" t="s">
+      <c r="B21" s="32" t="s">
         <v>133</v>
       </c>
-      <c r="C20" s="35" t="s">
+      <c r="C21" s="35" t="s">
         <v>111</v>
-      </c>
-      <c r="D20" s="34" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="37"/>
-      <c r="B21" s="32" t="s">
-        <v>132</v>
-      </c>
-      <c r="C21" s="35" t="s">
-        <v>112</v>
       </c>
       <c r="D21" s="34" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4">
       <c r="A22" s="37"/>
       <c r="B22" s="32" t="s">
+        <v>132</v>
+      </c>
+      <c r="C22" s="35" t="s">
+        <v>112</v>
+      </c>
+      <c r="D22" s="34" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="37"/>
+      <c r="B23" s="32" t="s">
         <v>124</v>
       </c>
-      <c r="C22" s="35" t="s">
+      <c r="C23" s="35" t="s">
         <v>126</v>
       </c>
-      <c r="D22" s="34"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="38"/>
-      <c r="B23" s="32" t="s">
+      <c r="D23" s="34"/>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="38"/>
+      <c r="B24" s="32" t="s">
         <v>127</v>
       </c>
-      <c r="C23" s="35" t="s">
+      <c r="C24" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="D23" s="34" t="s">
+      <c r="D24" s="34" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="C24" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="D24" s="28" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" ht="16.5">
       <c r="A25" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="D25" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>67</v>
+    <row r="26" spans="1:4" ht="16.5">
+      <c r="A26" s="6" t="s">
+        <v>5</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C26" s="25" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D26" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" ht="31.5">
       <c r="A27" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D27" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="6" t="s">
-        <v>5</v>
+    <row r="28" spans="1:4" ht="31.5">
+      <c r="A28" s="2" t="s">
+        <v>69</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C28" s="25" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D28" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A29" s="31" t="s">
+    <row r="29" spans="1:4">
+      <c r="A29" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B29" s="32" t="s">
-        <v>83</v>
-      </c>
-      <c r="C29" s="33" t="s">
-        <v>80</v>
-      </c>
-      <c r="D29" s="34" t="s">
+      <c r="B29" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C29" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="D29" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" ht="16.5">
       <c r="A30" s="31" t="s">
         <v>5</v>
       </c>
       <c r="B30" s="32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D30" s="34" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
+    <row r="31" spans="1:4" ht="16.5">
+      <c r="A31" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="B31" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="C31" s="33" t="s">
+        <v>81</v>
+      </c>
+      <c r="D31" s="34" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="16.5">
+      <c r="A32" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B32" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C31" s="25" t="s">
+      <c r="C32" s="25" t="s">
         <v>82</v>
-      </c>
-      <c r="D31" s="28" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A32" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="B32" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="C32" s="25" t="s">
-        <v>86</v>
       </c>
       <c r="D32" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A33" s="7" t="s">
-        <v>88</v>
+    <row r="33" spans="1:4" ht="16.5">
+      <c r="A33" s="2" t="s">
+        <v>87</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="C33" s="25" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D33" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A34" s="2" t="s">
-        <v>93</v>
+    <row r="34" spans="1:4" ht="16.5">
+      <c r="A34" s="7" t="s">
+        <v>88</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C34" s="25" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="D34" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="63" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
-        <v>5</v>
+    <row r="35" spans="1:4" ht="16.5">
+      <c r="A35" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="C35" s="25" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="D35" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" ht="63">
       <c r="A36" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>138</v>
+        <v>101</v>
       </c>
       <c r="C36" s="25" t="s">
-        <v>137</v>
+        <v>102</v>
       </c>
       <c r="D36" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" ht="31.5">
       <c r="A37" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B37" s="29" t="s">
-        <v>116</v>
+      <c r="B37" s="7" t="s">
+        <v>138</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="D37" s="3"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+      <c r="D37" s="28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
       <c r="A38" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B38" s="7" t="s">
-        <v>146</v>
+      <c r="B38" s="29" t="s">
+        <v>116</v>
       </c>
       <c r="C38" s="25" t="s">
-        <v>147</v>
-      </c>
-      <c r="D38" s="28" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+      <c r="D38" s="3"/>
+    </row>
+    <row r="39" spans="1:4">
       <c r="A39" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B39" s="29" t="s">
+      <c r="B39" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="C39" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="D39" s="28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B40" s="29" t="s">
         <v>114</v>
       </c>
-      <c r="C39" s="25" t="s">
+      <c r="C40" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="D39" s="3"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="31" t="s">
+      <c r="D40" s="3"/>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="B40" s="32" t="s">
+      <c r="B41" s="32" t="s">
         <v>115</v>
       </c>
-      <c r="C40" s="33" t="s">
+      <c r="C41" s="33" t="s">
         <v>105</v>
       </c>
-      <c r="D40" s="34" t="s">
+      <c r="D41" s="34" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B41" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="C41" s="25" t="s">
-        <v>119</v>
-      </c>
-      <c r="D41" s="28" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4">
       <c r="A42" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C42" s="25" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D42" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4">
       <c r="A43" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="C43" s="25" t="s">
-        <v>140</v>
+        <v>121</v>
       </c>
       <c r="D43" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4">
       <c r="A44" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C44" s="25" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D44" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4">
       <c r="A45" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C45" s="25" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D45" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4">
       <c r="A46" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C46" s="25" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D46" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4">
       <c r="A47" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="C47" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
+      </c>
+      <c r="C47" s="25" t="s">
+        <v>149</v>
       </c>
       <c r="D47" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A48" s="2" t="s">
-        <v>152</v>
+    <row r="48" spans="1:4" ht="31.5">
+      <c r="A48" s="6" t="s">
+        <v>5</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="C48" s="25" t="s">
-        <v>153</v>
+        <v>150</v>
+      </c>
+      <c r="C48" s="22" t="s">
+        <v>151</v>
       </c>
       <c r="D48" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A49" s="6" t="s">
-        <v>5</v>
+    <row r="49" spans="1:4" ht="31.5">
+      <c r="A49" s="2" t="s">
+        <v>152</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C49" s="25" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D49" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="2"/>
+    <row r="50" spans="1:4" ht="47.25">
+      <c r="A50" s="6" t="s">
+        <v>5</v>
+      </c>
       <c r="B50" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>157</v>
+        <v>156</v>
+      </c>
+      <c r="C50" s="25" t="s">
+        <v>155</v>
       </c>
       <c r="D50" s="28" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4">
       <c r="A51" s="2"/>
       <c r="B51" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D51" s="28" t="s">
         <v>34</v>
       </c>
     </row>
+    <row r="52" spans="1:4">
+      <c r="A52" s="2"/>
+      <c r="B52" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="D52" s="28" t="s">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="A20:A23"/>
-    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="A18:A20"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5201,7 +5223,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="12.25" style="11" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="66.875" style="12" customWidth="1"/>
@@ -5209,7 +5231,7 @@
     <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4">
       <c r="A1" s="13" t="s">
         <v>8</v>
       </c>
@@ -5223,7 +5245,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="69.75" customHeight="1">
       <c r="A2" s="9" t="s">
         <v>11</v>
       </c>
@@ -5237,7 +5259,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="69.75" customHeight="1">
       <c r="A3" s="9" t="s">
         <v>17</v>
       </c>
@@ -5249,7 +5271,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="69" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="69" customHeight="1">
       <c r="A4" s="9" t="s">
         <v>13</v>
       </c>
@@ -5263,7 +5285,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="35.25" customHeight="1">
       <c r="A5" s="9" t="s">
         <v>14</v>
       </c>
@@ -5277,7 +5299,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="213.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="213.75" customHeight="1">
       <c r="A6" s="9" t="s">
         <v>15</v>
       </c>
@@ -5299,7 +5321,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="24.5" style="11" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="61.875" style="12" customWidth="1"/>
@@ -5307,7 +5329,7 @@
     <col min="5" max="16384" width="9" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4">
       <c r="A1" s="13" t="s">
         <v>8</v>
       </c>
@@ -5321,7 +5343,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="252" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="252">
       <c r="A2" s="9" t="s">
         <v>16</v>
       </c>
@@ -5335,7 +5357,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="236.25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="236.25">
       <c r="A3" s="9" t="s">
         <v>36</v>
       </c>
@@ -5359,7 +5381,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="17.25" style="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="50.5" style="12" customWidth="1"/>
@@ -5368,7 +5390,7 @@
     <col min="5" max="16384" width="9" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4">
       <c r="A1" s="13" t="s">
         <v>8</v>
       </c>
@@ -5382,7 +5404,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="337.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="337.5" customHeight="1">
       <c r="A2" s="9" t="s">
         <v>12</v>
       </c>
@@ -5396,7 +5418,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="260.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="260.25" customHeight="1">
       <c r="A3" s="9" t="s">
         <v>17</v>
       </c>
@@ -5410,7 +5432,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="299.25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="299.25">
       <c r="A4" s="9" t="s">
         <v>18</v>
       </c>
@@ -5424,7 +5446,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="362.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="362.25" customHeight="1">
       <c r="A5" s="9" t="s">
         <v>19</v>
       </c>
@@ -5438,7 +5460,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="330.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="330.75">
       <c r="A6" s="9" t="s">
         <v>20</v>
       </c>
@@ -5452,7 +5474,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="378" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="378">
       <c r="A7" s="9" t="s">
         <v>21</v>
       </c>

</xml_diff>